<commit_message>
Fix Temple & Webster price note, document Australia Post sources, strengthen QA sheet
</commit_message>
<xml_diff>
--- a/Manoj_Kumar_Assessment_Workbook.xlsx
+++ b/Manoj_Kumar_Assessment_Workbook.xlsx
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="840" uniqueCount="583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="612">
   <si>
     <t xml:space="preserve">Market Research &amp; Data Analyst Assessment - Workbook</t>
   </si>
@@ -791,7 +791,7 @@
     <t xml:space="preserve">Current market price range (verified examples)</t>
   </si>
   <si>
-    <t xml:space="preserve">$69 (Bunnings Jack 160x80cm) to $84.95 (T&amp;W Gordo 160cm, was $124)</t>
+    <t xml:space="preserve">$69 (Bunnings Jack 160x80cm) to $84.95 (T&amp;W Gordo, from $84.95; its page shows a $84.95-$124 range across options)</t>
   </si>
   <si>
     <t xml:space="preserve">$42.85 (Kogan Beastie 104cm) to $150.99 (Kogan PaWz 138cm); Bunnings Alopet 142cm $82.43; Kmart Advwin 84cm $44.90</t>
@@ -902,7 +902,7 @@
     <t xml:space="preserve">https://www.bunnings.com.au/jack-1600-x-800mm-rectangular-raised-garden-bed_p0807491</t>
   </si>
   <si>
-    <t xml:space="preserve">Temple &amp; Webster - Living Fusion Gordo Galvanised Steel Raised Garden Bed (160cm)</t>
+    <t xml:space="preserve">Temple &amp; Webster - Living Fusion Gordo Galvanised Steel Raised Garden Bed (from $84.95; page shows a $84.95-$124 range across size/colour options, not a was-price)</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.templeandwebster.com.au/Gordo-Galvanised-Steel-Raised-Garden-Bed-OIKT1274.html</t>
@@ -1316,6 +1316,9 @@
     <t xml:space="preserve">All accessed 8 Oct 2026 unless stated. 'Opened' = read on the live page by me; 'Fetched' = read via the page-fetch tool.</t>
   </si>
   <si>
+    <t xml:space="preserve">Evidence class: PRIMARY = read on the original page or official report. SECONDARY = a third party reporting someone else's figure. No figure in the answers rests on a search snippet alone. Potential selling prices and risk statements in Q5 are analyst INFERENCE and are labelled as such in the answers.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Source ID</t>
   </si>
   <si>
@@ -1331,6 +1334,9 @@
     <t xml:space="preserve">Access date</t>
   </si>
   <si>
+    <t xml:space="preserve">Evidence class</t>
+  </si>
+  <si>
     <t xml:space="preserve">S01</t>
   </si>
   <si>
@@ -1346,6 +1352,9 @@
     <t xml:space="preserve">Retailer product page (opened in Chrome)</t>
   </si>
   <si>
+    <t xml:space="preserve">PRIMARY</t>
+  </si>
+  <si>
     <t xml:space="preserve">S02</t>
   </si>
   <si>
@@ -1637,12 +1646,66 @@
     <t xml:space="preserve">Official industry report (fetched)</t>
   </si>
   <si>
-    <t xml:space="preserve">A press report quotes $11.4b for Home &amp; Garden from the main report; not reconciled, so only the category PDF figure is used.</t>
+    <t xml:space="preserve">Three press/industry-blog articles (S35-S37) quote $11.4b for Home &amp; Garden and attribute it to the main report. Not reconciled, so the $9.9b read in this PDF is used and the conflict is stated in the answers. The PDF itself credits CommBank iQ and points to p.38 of the main report, which was not opened.</t>
   </si>
   <si>
     <t xml:space="preserve">S35</t>
   </si>
   <si>
+    <t xml:space="preserve">Press: Parcel &amp; Postal Technology International</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quotes Home &amp; Garden online spend A$11.4bn (2025) from the Australia Post report; Fashion A$11.6bn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.parcelandpostaltechnologyinternational.com/news/e-commerce/australian-online-spending-reaches-a82-6bn-in-2025.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trade press article (fetched)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secondary source; conflicts with the $9.9b in the category PDF (S34).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SECONDARY</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S36</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Press: IPC (International Post Corporation)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Quotes Home and Garden $11.4 billion; Online Marketplaces $18.9b; Fashion $11.6b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.ipc.be/news-portal/e-commerce/2026/03/18/16/03/aussies-add-82-6-billion-to-cart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secondary source; conflicts with S34.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S37</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Blog: eightx.co</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lists Home &amp; Garden $11.4B, +10.5% YoY, citing the Australia Post 2026 report</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://eightx.co/blog/australian-online-retail-category-share-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Industry blog (fetched)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Secondary source; weakest of the three. Conflicts with S34 on both value and growth (+10.5% vs +9.9%).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S38</t>
+  </si>
+  <si>
     <t xml:space="preserve">Australia Post - Pet products</t>
   </si>
   <si>
@@ -1652,7 +1715,7 @@
     <t xml:space="preserve">https://auspost.com.au/content/dam/auspost_corp/media/documents/australia-post-ecommerce-report-2026-pet-products.pdf</t>
   </si>
   <si>
-    <t xml:space="preserve">S36</t>
+    <t xml:space="preserve">S39</t>
   </si>
   <si>
     <t xml:space="preserve">Q7</t>
@@ -1670,7 +1733,7 @@
     <t xml:space="preserve">Official industry report page (fetched)</t>
   </si>
   <si>
-    <t xml:space="preserve">S37</t>
+    <t xml:space="preserve">S40</t>
   </si>
   <si>
     <t xml:space="preserve">Australia Post eCommerce trends (FY26 Q4 update)</t>
@@ -1682,7 +1745,7 @@
     <t xml:space="preserve">https://auspost.com.au/business/marketing-and-communications/access-data-and-insights/ecommerce-trends</t>
   </si>
   <si>
-    <t xml:space="preserve">S38</t>
+    <t xml:space="preserve">S41</t>
   </si>
   <si>
     <t xml:space="preserve">Q7/Q13</t>
@@ -1700,7 +1763,7 @@
     <t xml:space="preserve">Government statistics (fetched)</t>
   </si>
   <si>
-    <t xml:space="preserve">S39</t>
+    <t xml:space="preserve">S42</t>
   </si>
   <si>
     <t xml:space="preserve">Amazon AU Best Sellers</t>
@@ -1718,7 +1781,7 @@
     <t xml:space="preserve">Rank only; no unit sales published.</t>
   </si>
   <si>
-    <t xml:space="preserve">S40</t>
+    <t xml:space="preserve">S43</t>
   </si>
   <si>
     <t xml:space="preserve">Office chair/garden/pet category pages with 'Don't Pay' reference prices and seller names</t>
@@ -1730,7 +1793,7 @@
     <t xml:space="preserve">Retailer (opened in Chrome)</t>
   </si>
   <si>
-    <t xml:space="preserve">S41</t>
+    <t xml:space="preserve">S44</t>
   </si>
   <si>
     <t xml:space="preserve">Q13</t>
@@ -1779,6 +1842,30 @@
   </si>
   <si>
     <t xml:space="preserve">Sources: at least 30 rows registered</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q6: net profit rounds to 17.45 and net margin to 11.6%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q6: total listed costs = 22.50 (3% x 149.95 + 8 + 10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q8: conversion Jan-Apr = 2.00%, 1.75%, 1.37%, 1.05% (typed independently)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q8: conversion recomputed from raw inputs (orders / visitors) matches column E</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q9: stage rates = 5%, 20%, 20% and overall 0.20% (typed independently)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q4: all 15 prices recompute the same median via a second route (SUMPRODUCT rank)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Q4: 15 distinct product IDs (no duplicated records)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sources: every source row has an https URL</t>
   </si>
   <si>
     <t xml:space="preserve">Overall</t>
@@ -1958,7 +2045,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="41">
+  <cellXfs count="43">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -2011,7 +2098,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2092,6 +2179,14 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2426,7 +2521,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:B17"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -2560,7 +2655,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -2571,9 +2666,9 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H45"/>
+  <dimension ref="A1:I48"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="9"/>
@@ -2583,6 +2678,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="13"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="50"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="15"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2595,1025 +2691,1253 @@
         <v>426</v>
       </c>
     </row>
+    <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="13" t="s">
+        <v>427</v>
+      </c>
+      <c r="B3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="13"/>
+      <c r="F3" s="13"/>
+      <c r="G3" s="13"/>
+      <c r="H3" s="13"/>
+    </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="5" t="s">
-        <v>427</v>
+        <v>428</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>356</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>428</v>
+        <v>429</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>429</v>
+        <v>430</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>285</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>430</v>
+        <v>431</v>
       </c>
       <c r="G4" s="5" t="s">
-        <v>431</v>
+        <v>432</v>
       </c>
       <c r="H4" s="5" t="s">
         <v>207</v>
       </c>
+      <c r="I4" s="5" t="s">
+        <v>433</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>432</v>
+        <v>434</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>434</v>
+        <v>436</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>435</v>
+        <v>437</v>
       </c>
       <c r="E5" s="25" t="s">
         <v>122</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G5" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H5" s="4"/>
+      <c r="I5" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>437</v>
+        <v>440</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>438</v>
+        <v>441</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>439</v>
+        <v>442</v>
       </c>
       <c r="E6" s="25" t="s">
         <v>128</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G6" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H6" s="4"/>
+      <c r="I6" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>440</v>
+        <v>443</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>441</v>
+        <v>444</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>442</v>
+        <v>445</v>
       </c>
       <c r="E7" s="25" t="s">
         <v>135</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G7" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H7" s="4"/>
+      <c r="I7" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>443</v>
+        <v>446</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>444</v>
+        <v>447</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>445</v>
+        <v>448</v>
       </c>
       <c r="E8" s="25" t="s">
         <v>141</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G8" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H8" s="4"/>
+      <c r="I8" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>446</v>
+        <v>449</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>447</v>
+        <v>450</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>448</v>
+        <v>451</v>
       </c>
       <c r="E9" s="25" t="s">
         <v>146</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G9" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H9" s="4"/>
+      <c r="I9" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>449</v>
+        <v>452</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>450</v>
+        <v>453</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>451</v>
+        <v>454</v>
       </c>
       <c r="E10" s="25" t="s">
         <v>152</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G10" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H10" s="4"/>
+      <c r="I10" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>452</v>
+        <v>455</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>453</v>
+        <v>456</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>454</v>
+        <v>457</v>
       </c>
       <c r="E11" s="25" t="s">
         <v>158</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G11" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H11" s="4"/>
+      <c r="I11" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>455</v>
+        <v>458</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>456</v>
+        <v>459</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>457</v>
+        <v>460</v>
       </c>
       <c r="E12" s="25" t="s">
         <v>163</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G12" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H12" s="4"/>
+      <c r="I12" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>458</v>
+        <v>461</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>459</v>
+        <v>462</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>460</v>
+        <v>463</v>
       </c>
       <c r="E13" s="25" t="s">
         <v>167</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G13" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H13" s="4"/>
+      <c r="I13" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>461</v>
+        <v>464</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>462</v>
+        <v>465</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>463</v>
+        <v>466</v>
       </c>
       <c r="E14" s="25" t="s">
         <v>175</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G14" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H14" s="4"/>
+      <c r="I14" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>464</v>
+        <v>467</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>465</v>
+        <v>468</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>466</v>
+        <v>469</v>
       </c>
       <c r="E15" s="25" t="s">
         <v>180</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G15" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H15" s="4"/>
+      <c r="I15" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>467</v>
+        <v>470</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>468</v>
+        <v>471</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>469</v>
+        <v>472</v>
       </c>
       <c r="E16" s="25" t="s">
         <v>187</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G16" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H16" s="4"/>
+      <c r="I16" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>470</v>
+        <v>473</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>471</v>
+        <v>474</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>472</v>
+        <v>475</v>
       </c>
       <c r="E17" s="25" t="s">
         <v>195</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G17" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H17" s="4"/>
+      <c r="I17" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>473</v>
+        <v>476</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>474</v>
+        <v>477</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>475</v>
+        <v>478</v>
       </c>
       <c r="E18" s="25" t="s">
         <v>200</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G18" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H18" s="4"/>
+      <c r="I18" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>476</v>
+        <v>479</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>477</v>
+        <v>480</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>478</v>
+        <v>481</v>
       </c>
       <c r="E19" s="25" t="s">
         <v>205</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>436</v>
+        <v>438</v>
       </c>
       <c r="G19" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H19" s="4"/>
+      <c r="I19" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>479</v>
+        <v>482</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C20" s="4" t="s">
         <v>114</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>480</v>
+        <v>483</v>
       </c>
       <c r="E20" s="25" t="s">
-        <v>481</v>
+        <v>484</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="G20" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H20" s="4"/>
+      <c r="I20" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>483</v>
+        <v>486</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C21" s="4" t="s">
         <v>138</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>484</v>
+        <v>487</v>
       </c>
       <c r="E21" s="25" t="s">
+        <v>488</v>
+      </c>
+      <c r="F21" s="4" t="s">
         <v>485</v>
-      </c>
-      <c r="F21" s="4" t="s">
-        <v>482</v>
       </c>
       <c r="G21" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H21" s="4"/>
+      <c r="I21" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>486</v>
+        <v>489</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C22" s="4" t="s">
         <v>155</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>487</v>
+        <v>490</v>
       </c>
       <c r="E22" s="25" t="s">
-        <v>488</v>
+        <v>491</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>482</v>
+        <v>485</v>
       </c>
       <c r="G22" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H22" s="4"/>
+      <c r="I22" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>489</v>
+        <v>492</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C23" s="4" t="s">
         <v>170</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>490</v>
+        <v>493</v>
       </c>
       <c r="E23" s="25" t="s">
-        <v>491</v>
+        <v>494</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>492</v>
+        <v>495</v>
       </c>
       <c r="G23" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H23" s="4"/>
+      <c r="I23" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>493</v>
+        <v>496</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>433</v>
+        <v>435</v>
       </c>
       <c r="C24" s="4" t="s">
         <v>190</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>494</v>
+        <v>497</v>
       </c>
       <c r="E24" s="25" t="s">
+        <v>498</v>
+      </c>
+      <c r="F24" s="4" t="s">
         <v>495</v>
-      </c>
-      <c r="F24" s="4" t="s">
-        <v>492</v>
       </c>
       <c r="G24" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H24" s="4"/>
+      <c r="I24" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>496</v>
+        <v>499</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C25" s="4" t="s">
         <v>287</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>498</v>
+        <v>501</v>
       </c>
       <c r="E25" s="25" t="s">
         <v>288</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G25" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H25" s="4"/>
-    </row>
-    <row r="26" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I25" s="4" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="B26" s="4" t="s">
         <v>500</v>
-      </c>
-      <c r="B26" s="4" t="s">
-        <v>497</v>
       </c>
       <c r="C26" s="4" t="s">
         <v>289</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>501</v>
+        <v>504</v>
       </c>
       <c r="E26" s="25" t="s">
         <v>290</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G26" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H26" s="4"/>
+      <c r="I26" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>502</v>
+        <v>505</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C27" s="4" t="s">
         <v>292</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>503</v>
+        <v>506</v>
       </c>
       <c r="E27" s="25" t="s">
         <v>293</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G27" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H27" s="4"/>
+      <c r="I27" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>504</v>
+        <v>507</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C28" s="4" t="s">
         <v>294</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>505</v>
+        <v>508</v>
       </c>
       <c r="E28" s="25" t="s">
         <v>295</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G28" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H28" s="4"/>
+      <c r="I28" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>506</v>
+        <v>509</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C29" s="4" t="s">
         <v>296</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>507</v>
+        <v>510</v>
       </c>
       <c r="E29" s="25" t="s">
         <v>297</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G29" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H29" s="4"/>
+      <c r="I29" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>508</v>
+        <v>511</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C30" s="4" t="s">
         <v>298</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>509</v>
+        <v>512</v>
       </c>
       <c r="E30" s="25" t="s">
         <v>299</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G30" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H30" s="4"/>
+      <c r="I30" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>510</v>
+        <v>513</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C31" s="4" t="s">
         <v>301</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>511</v>
+        <v>514</v>
       </c>
       <c r="E31" s="25" t="s">
         <v>302</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G31" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H31" s="4"/>
+      <c r="I31" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>512</v>
+        <v>515</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C32" s="4" t="s">
         <v>303</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>513</v>
+        <v>516</v>
       </c>
       <c r="E32" s="25" t="s">
         <v>304</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G32" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H32" s="4"/>
+      <c r="I32" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>514</v>
+        <v>517</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C33" s="4" t="s">
         <v>305</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>515</v>
+        <v>518</v>
       </c>
       <c r="E33" s="25" t="s">
         <v>304</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G33" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H33" s="4"/>
+      <c r="I33" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>516</v>
+        <v>519</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C34" s="4" t="s">
         <v>306</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>517</v>
+        <v>520</v>
       </c>
       <c r="E34" s="25" t="s">
         <v>304</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G34" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H34" s="4"/>
+      <c r="I34" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C35" s="4" t="s">
         <v>307</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>519</v>
+        <v>522</v>
       </c>
       <c r="E35" s="25" t="s">
         <v>304</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G35" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H35" s="4"/>
+      <c r="I35" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>520</v>
+        <v>523</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C36" s="4" t="s">
         <v>308</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>521</v>
+        <v>524</v>
       </c>
       <c r="E36" s="25" t="s">
         <v>304</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>499</v>
+        <v>502</v>
       </c>
       <c r="G36" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H36" s="4"/>
+      <c r="I36" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>522</v>
+        <v>525</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>497</v>
+        <v>500</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>524</v>
+        <v>527</v>
       </c>
       <c r="E37" s="25" t="s">
-        <v>525</v>
+        <v>528</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>526</v>
+        <v>529</v>
       </c>
       <c r="G37" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H37" s="4" t="s">
-        <v>527</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>530</v>
+      </c>
+      <c r="I37" s="4" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>528</v>
+        <v>531</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>530</v>
+        <v>533</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>531</v>
+        <v>534</v>
       </c>
       <c r="E38" s="25" t="s">
-        <v>532</v>
+        <v>535</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>533</v>
+        <v>536</v>
       </c>
       <c r="G38" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>534</v>
+        <v>537</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>535</v>
+        <v>538</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>529</v>
+        <v>532</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>536</v>
+        <v>539</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>537</v>
+        <v>540</v>
       </c>
       <c r="E39" s="25" t="s">
-        <v>538</v>
+        <v>541</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>533</v>
+        <v>542</v>
       </c>
       <c r="G39" s="26" t="n">
         <v>46303</v>
       </c>
-      <c r="H39" s="4"/>
-    </row>
-    <row r="40" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H39" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>544</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>539</v>
+        <v>545</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>541</v>
+        <v>546</v>
       </c>
       <c r="D40" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="E40" s="25" t="s">
+        <v>548</v>
+      </c>
+      <c r="F40" s="4" t="s">
         <v>542</v>
-      </c>
-      <c r="E40" s="25" t="s">
-        <v>543</v>
-      </c>
-      <c r="F40" s="4" t="s">
-        <v>544</v>
       </c>
       <c r="G40" s="26" t="n">
         <v>46303</v>
       </c>
-      <c r="H40" s="4"/>
+      <c r="H40" s="4" t="s">
+        <v>549</v>
+      </c>
+      <c r="I40" s="4" t="s">
+        <v>544</v>
+      </c>
     </row>
     <row r="41" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="4" t="s">
-        <v>545</v>
+        <v>550</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>540</v>
+        <v>532</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>546</v>
+        <v>551</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>547</v>
+        <v>552</v>
       </c>
       <c r="E41" s="25" t="s">
-        <v>548</v>
+        <v>553</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>544</v>
+        <v>554</v>
       </c>
       <c r="G41" s="26" t="n">
         <v>46303</v>
       </c>
-      <c r="H41" s="4"/>
+      <c r="H41" s="4" t="s">
+        <v>555</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>544</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>549</v>
+        <v>556</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>550</v>
+        <v>532</v>
       </c>
       <c r="C42" s="4" t="s">
-        <v>551</v>
+        <v>557</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>552</v>
+        <v>558</v>
       </c>
       <c r="E42" s="25" t="s">
-        <v>553</v>
+        <v>559</v>
       </c>
       <c r="F42" s="4" t="s">
-        <v>554</v>
+        <v>536</v>
       </c>
       <c r="G42" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H42" s="4"/>
-    </row>
-    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="I42" s="4" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="4" t="s">
-        <v>555</v>
+        <v>560</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>550</v>
+        <v>561</v>
       </c>
       <c r="C43" s="4" t="s">
-        <v>556</v>
+        <v>562</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>557</v>
+        <v>563</v>
       </c>
       <c r="E43" s="25" t="s">
-        <v>558</v>
+        <v>564</v>
       </c>
       <c r="F43" s="4" t="s">
-        <v>559</v>
+        <v>565</v>
       </c>
       <c r="G43" s="26" t="n">
         <v>46303</v>
       </c>
-      <c r="H43" s="4" t="s">
-        <v>560</v>
+      <c r="H43" s="4"/>
+      <c r="I43" s="4" t="s">
+        <v>439</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="4" t="s">
+        <v>566</v>
+      </c>
+      <c r="B44" s="4" t="s">
         <v>561</v>
       </c>
-      <c r="B44" s="4" t="s">
-        <v>540</v>
-      </c>
       <c r="C44" s="4" t="s">
-        <v>170</v>
+        <v>567</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>562</v>
+        <v>568</v>
       </c>
       <c r="E44" s="25" t="s">
-        <v>563</v>
+        <v>569</v>
       </c>
       <c r="F44" s="4" t="s">
-        <v>564</v>
+        <v>565</v>
       </c>
       <c r="G44" s="26" t="n">
         <v>46303</v>
       </c>
       <c r="H44" s="4"/>
+      <c r="I44" s="4" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="4" t="s">
-        <v>565</v>
+        <v>570</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>566</v>
+        <v>571</v>
       </c>
       <c r="C45" s="4" t="s">
-        <v>114</v>
+        <v>572</v>
       </c>
       <c r="D45" s="4" t="s">
-        <v>567</v>
+        <v>573</v>
       </c>
       <c r="E45" s="25" t="s">
-        <v>481</v>
+        <v>574</v>
       </c>
       <c r="F45" s="4" t="s">
-        <v>482</v>
+        <v>575</v>
       </c>
       <c r="G45" s="26" t="n">
         <v>46303</v>
       </c>
-      <c r="H45" s="4" t="s">
-        <v>568</v>
+      <c r="H45" s="4"/>
+      <c r="I45" s="4" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
+        <v>576</v>
+      </c>
+      <c r="B46" s="4" t="s">
+        <v>571</v>
+      </c>
+      <c r="C46" s="4" t="s">
+        <v>577</v>
+      </c>
+      <c r="D46" s="4" t="s">
+        <v>578</v>
+      </c>
+      <c r="E46" s="25" t="s">
+        <v>579</v>
+      </c>
+      <c r="F46" s="4" t="s">
+        <v>580</v>
+      </c>
+      <c r="G46" s="26" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H46" s="4" t="s">
+        <v>581</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="s">
+        <v>582</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>561</v>
+      </c>
+      <c r="C47" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="D47" s="4" t="s">
+        <v>583</v>
+      </c>
+      <c r="E47" s="25" t="s">
+        <v>584</v>
+      </c>
+      <c r="F47" s="4" t="s">
+        <v>585</v>
+      </c>
+      <c r="G47" s="26" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H47" s="4"/>
+      <c r="I47" s="4" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="s">
+        <v>586</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>587</v>
+      </c>
+      <c r="C48" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="D48" s="4" t="s">
+        <v>588</v>
+      </c>
+      <c r="E48" s="25" t="s">
+        <v>484</v>
+      </c>
+      <c r="F48" s="4" t="s">
+        <v>485</v>
+      </c>
+      <c r="G48" s="26" t="n">
+        <v>46303</v>
+      </c>
+      <c r="H48" s="4" t="s">
+        <v>589</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>439</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A3:H3"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="E5" r:id="rId1" display="https://www.kmart.com.au/product/boucle-home-office-chair-43228386/"/>
     <hyperlink ref="E6" r:id="rId2" display="https://www.kmart.com.au/product/sky-office-chair-43682737/"/>
@@ -3649,17 +3973,20 @@
     <hyperlink ref="E36" r:id="rId32" display="https://www.bunnings.com.au/products/outdoor-living/outdoor-furniture/outdoor-storage/outdoor-storage-boxes"/>
     <hyperlink ref="E37" r:id="rId33" display="https://trends.google.com/trends/explore?date=today%205-y&amp;geo=AU&amp;q=raised%20garden%20bed,outdoor%20storage%20box,cat%20tree&amp;hl=en-AU"/>
     <hyperlink ref="E38" r:id="rId34" display="https://auspost.com.au/content/dam/auspost_corp/media/documents/australia-post-ecommerce-report-2026-home-garden.pdf"/>
-    <hyperlink ref="E39" r:id="rId35" display="https://auspost.com.au/content/dam/auspost_corp/media/documents/australia-post-ecommerce-report-2026-pet-products.pdf"/>
-    <hyperlink ref="E40" r:id="rId36" display="https://auspost.com.au/business/ecommerce/ecommerce-report"/>
-    <hyperlink ref="E41" r:id="rId37" display="https://auspost.com.au/business/marketing-and-communications/access-data-and-insights/ecommerce-trends"/>
-    <hyperlink ref="E42" r:id="rId38" display="https://www.abs.gov.au/media-centre/media-releases/household-spending-unchanged-august"/>
-    <hyperlink ref="E43" r:id="rId39" display="https://www.amazon.com.au/gp/bestsellers/home/4975214051"/>
-    <hyperlink ref="E44" r:id="rId40" display="https://www.kogan.com/au/c/garden-beds/"/>
-    <hyperlink ref="E45" r:id="rId41" display="https://www.kmart.com.au/search/?searchTerm=office%20chair"/>
+    <hyperlink ref="E39" r:id="rId35" display="https://www.parcelandpostaltechnologyinternational.com/news/e-commerce/australian-online-spending-reaches-a82-6bn-in-2025.html"/>
+    <hyperlink ref="E40" r:id="rId36" display="https://www.ipc.be/news-portal/e-commerce/2026/03/18/16/03/aussies-add-82-6-billion-to-cart"/>
+    <hyperlink ref="E41" r:id="rId37" display="https://eightx.co/blog/australian-online-retail-category-share-2026"/>
+    <hyperlink ref="E42" r:id="rId38" display="https://auspost.com.au/content/dam/auspost_corp/media/documents/australia-post-ecommerce-report-2026-pet-products.pdf"/>
+    <hyperlink ref="E43" r:id="rId39" display="https://auspost.com.au/business/ecommerce/ecommerce-report"/>
+    <hyperlink ref="E44" r:id="rId40" display="https://auspost.com.au/business/marketing-and-communications/access-data-and-insights/ecommerce-trends"/>
+    <hyperlink ref="E45" r:id="rId41" display="https://www.abs.gov.au/media-centre/media-releases/household-spending-unchanged-august"/>
+    <hyperlink ref="E46" r:id="rId42" display="https://www.amazon.com.au/gp/bestsellers/home/4975214051"/>
+    <hyperlink ref="E47" r:id="rId43" display="https://www.kogan.com/au/c/garden-beds/"/>
+    <hyperlink ref="E48" r:id="rId44" display="https://www.kmart.com.au/search/?searchTerm=office%20chair"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3670,9 +3997,9 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="60"/>
@@ -3681,12 +4008,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>569</v>
+        <v>590</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="5" t="s">
-        <v>570</v>
+        <v>591</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>336</v>
@@ -3694,7 +4021,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>571</v>
+        <v>592</v>
       </c>
       <c r="B4" s="10" t="str">
         <f aca="false">IF(SUM(Q1_Profit!D5:D9)=SUM(Q1_Profit!C5:C9)-SUM(Q1_Profit!B5:B9),"PASS","FAIL")</f>
@@ -3703,7 +4030,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>572</v>
+        <v>593</v>
       </c>
       <c r="B5" s="10" t="str">
         <f aca="false">IF(Q1_Profit!B11="Bedside Table","PASS","FAIL")</f>
@@ -3712,7 +4039,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>573</v>
+        <v>594</v>
       </c>
       <c r="B6" s="10" t="str">
         <f aca="false">IF(COUNTA(Q4_Competitors!A5:A19)=15,"PASS","FAIL")</f>
@@ -3721,7 +4048,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>574</v>
+        <v>595</v>
       </c>
       <c r="B7" s="10" t="str">
         <f aca="false">IF(MIN(Q4_Summary!B5:B9)&gt;=3,"PASS","FAIL")</f>
@@ -3730,7 +4057,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>575</v>
+        <v>596</v>
       </c>
       <c r="B8" s="10" t="str">
         <f aca="false">IF(COUNTIF(Q4_Competitors!O5:O19,"https://*")=15,"PASS","FAIL")</f>
@@ -3739,7 +4066,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>576</v>
+        <v>597</v>
       </c>
       <c r="B9" s="10" t="str">
         <f aca="false">IF(COUNT(Q4_Competitors!G5:G19)=15,"PASS","FAIL")</f>
@@ -3748,7 +4075,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>577</v>
+        <v>598</v>
       </c>
       <c r="B10" s="10" t="str">
         <f aca="false">IF(Q6_Profitability!C22="MATCHES row 18","PASS","FAIL")</f>
@@ -3757,7 +4084,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>578</v>
+        <v>599</v>
       </c>
       <c r="B11" s="10" t="str">
         <f aca="false">IF(ROUND(Q6_Profitability!B12,2)=39.95,"PASS","FAIL")</f>
@@ -3766,7 +4093,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>579</v>
+        <v>600</v>
       </c>
       <c r="B12" s="10" t="str">
         <f aca="false">IF(AND(Q8_Sales!F5=150,Q8_Sales!F6=150,Q8_Sales!F7=150,Q8_Sales!F8=150),"PASS","FAIL")</f>
@@ -3775,7 +4102,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>580</v>
+        <v>601</v>
       </c>
       <c r="B13" s="10" t="str">
         <f aca="false">IF(Q9_Funnel!B17="OK","PASS","FAIL")</f>
@@ -3784,26 +4111,98 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>581</v>
+        <v>602</v>
       </c>
       <c r="B14" s="10" t="str">
         <f aca="false">IF(COUNTA(Sources!A5:A200)&gt;=30,"PASS","FAIL")</f>
         <v>PASS</v>
       </c>
     </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>603</v>
+      </c>
+      <c r="B15" s="10" t="str">
+        <f aca="false">IF(AND(ROUND(Q6_Profitability!B18,2)=17.45,ROUND(Q6_Profitability!B19,3)=0.116),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>582</v>
+      <c r="A16" s="4" t="s">
+        <v>604</v>
       </c>
       <c r="B16" s="10" t="str">
-        <f aca="false">IF(COUNTIF(B4:B14,"PASS")=11,"ALL PASS","REVIEW")</f>
+        <f aca="false">IF(ROUND(Q6_Profitability!B17,2)=22.5,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>605</v>
+      </c>
+      <c r="B17" s="10" t="str">
+        <f aca="false">IF(AND(ROUND(Q8_Sales!E5,4)=0.02,ROUND(Q8_Sales!E6,4)=0.0175,ROUND(Q8_Sales!E7,4)=0.0137,ROUND(Q8_Sales!E8,4)=0.0105),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>606</v>
+      </c>
+      <c r="B18" s="10" t="str">
+        <f aca="false">IF(ABS(Q8_Sales!E8-Q8_Sales!C8/Q8_Sales!B8)+ABS(Q8_Sales!E5-Q8_Sales!C5/Q8_Sales!B5)&lt;0.0000001,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>607</v>
+      </c>
+      <c r="B19" s="10" t="str">
+        <f aca="false">IF(AND(ROUND(Q9_Funnel!D11,4)=0.05,ROUND(Q9_Funnel!D12,4)=0.2,ROUND(Q9_Funnel!D13,4)=0.2,ROUND(Q9_Funnel!D14,4)=0.002),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>608</v>
+      </c>
+      <c r="B20" s="10" t="str">
+        <f aca="false">IF(COUNTIF(Q4_Competitors!G5:G19,"&lt;"&amp;Q4_Summary!D10)=7,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="4" t="s">
+        <v>609</v>
+      </c>
+      <c r="B21" s="10" t="str">
+        <f aca="false">IF(SUMPRODUCT(1/COUNTIF(Q4_Competitors!A5:A19,Q4_Competitors!A5:A19))=15,"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="4" t="s">
+        <v>610</v>
+      </c>
+      <c r="B22" s="10" t="str">
+        <f aca="false">IF(COUNTIF(Sources!E5:E200,"https://*")=COUNTA(Sources!A5:A200),"PASS","FAIL")</f>
+        <v>PASS</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
+        <v>611</v>
+      </c>
+      <c r="B24" s="10" t="str">
+        <f aca="false">IF(COUNTIF(B4:B22,"PASS")=19,"ALL PASS","REVIEW")</f>
         <v>ALL PASS</v>
       </c>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -3814,7 +4213,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:H16"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -4056,20 +4455,38 @@
         <v>0.315068493150685</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
         <v>48</v>
       </c>
-    </row>
-    <row r="16" customFormat="false" ht="79.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+    </row>
+    <row r="16" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
         <v>49</v>
       </c>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="13"/>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13"/>
+      <c r="H16" s="13"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A16:H16"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -4080,7 +4497,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:E24"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -4397,15 +4814,22 @@
         <v>91</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="158.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="13" t="s">
         <v>92</v>
       </c>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A24:E24"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -4416,7 +4840,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:R27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -5394,30 +5818,65 @@
         <v>207</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2" t="s">
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
         <v>208</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="s">
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+    </row>
+    <row r="23" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
         <v>209</v>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
+    </row>
+    <row r="24" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="13" t="s">
         <v>210</v>
       </c>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="2" t="s">
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="13"/>
+      <c r="F24" s="13"/>
+      <c r="G24" s="13"/>
+      <c r="H24" s="13"/>
+    </row>
+    <row r="25" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="s">
         <v>211</v>
       </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="2" t="s">
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="13"/>
+      <c r="F25" s="13"/>
+      <c r="G25" s="13"/>
+      <c r="H25" s="13"/>
+    </row>
+    <row r="26" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="s">
         <v>212</v>
       </c>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="13"/>
+      <c r="F26" s="13"/>
+      <c r="G26" s="13"/>
+      <c r="H26" s="13"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="2" t="s">
@@ -5426,6 +5885,13 @@
     </row>
   </sheetData>
   <autoFilter ref="A4:R19"/>
+  <mergeCells count="5">
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A24:H24"/>
+    <mergeCell ref="A25:H25"/>
+    <mergeCell ref="A26:H26"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="O5" r:id="rId1" display="https://www.kmart.com.au/product/boucle-home-office-chair-43228386/"/>
     <hyperlink ref="O6" r:id="rId2" display="https://www.kmart.com.au/product/sky-office-chair-43682737/"/>
@@ -5445,7 +5911,7 @@
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -5457,7 +5923,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:J32"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -5940,7 +6406,7 @@
       </c>
     </row>
     <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="13" t="s">
+      <c r="A22" s="34" t="s">
         <v>231</v>
       </c>
     </row>
@@ -6014,7 +6480,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -6025,7 +6491,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:G49"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -6240,7 +6706,7 @@
         <v>288</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
         <v>286</v>
       </c>
@@ -6250,8 +6716,8 @@
       <c r="C18" s="21" t="n">
         <v>84.95</v>
       </c>
-      <c r="D18" s="22" t="n">
-        <v>124</v>
+      <c r="D18" s="22" t="s">
+        <v>120</v>
       </c>
       <c r="E18" s="27" t="n">
         <v>4.6</v>
@@ -6563,10 +7029,16 @@
         <v>130.475</v>
       </c>
     </row>
-    <row r="37" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="29" t="s">
+    <row r="37" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="35" t="s">
         <v>313</v>
       </c>
+      <c r="B37" s="35"/>
+      <c r="C37" s="35"/>
+      <c r="D37" s="35"/>
+      <c r="E37" s="35"/>
+      <c r="F37" s="35"/>
+      <c r="G37" s="35"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="5" t="s">
@@ -6583,7 +7055,7 @@
       <c r="A39" s="4" t="s">
         <v>316</v>
       </c>
-      <c r="B39" s="34" t="n">
+      <c r="B39" s="36" t="n">
         <v>0.03</v>
       </c>
       <c r="C39" s="4" t="s">
@@ -6616,7 +7088,7 @@
       <c r="A42" s="4" t="s">
         <v>322</v>
       </c>
-      <c r="B42" s="34" t="n">
+      <c r="B42" s="36" t="n">
         <v>0.15</v>
       </c>
       <c r="C42" s="4" t="s">
@@ -6685,12 +7157,22 @@
         <v>19.35</v>
       </c>
     </row>
-    <row r="49" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="49" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="13" t="s">
         <v>329</v>
       </c>
+      <c r="B49" s="13"/>
+      <c r="C49" s="13"/>
+      <c r="D49" s="13"/>
+      <c r="E49" s="13"/>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A49:G49"/>
+  </mergeCells>
   <hyperlinks>
     <hyperlink ref="G17" r:id="rId1" display="https://www.bunnings.com.au/jack-1600-x-800mm-rectangular-raised-garden-bed_p0807491"/>
     <hyperlink ref="G18" r:id="rId2" display="https://www.templeandwebster.com.au/Gordo-Galvanised-Steel-Raised-Garden-Bed-OIKT1274.html"/>
@@ -6707,7 +7189,7 @@
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -6718,7 +7200,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:C43"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -6766,7 +7248,7 @@
       <c r="A7" s="4" t="s">
         <v>334</v>
       </c>
-      <c r="B7" s="34" t="n">
+      <c r="B7" s="36" t="n">
         <v>0.03</v>
       </c>
     </row>
@@ -6801,7 +7283,7 @@
       <c r="A12" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="B12" s="35" t="n">
+      <c r="B12" s="37" t="n">
         <f aca="false">B5-B6</f>
         <v>39.95</v>
       </c>
@@ -6813,7 +7295,7 @@
       <c r="A13" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="B13" s="36" t="n">
+      <c r="B13" s="38" t="n">
         <f aca="false">B12/B5</f>
         <v>0.266422140713571</v>
       </c>
@@ -6873,7 +7355,7 @@
       <c r="A18" s="3" t="s">
         <v>349</v>
       </c>
-      <c r="B18" s="35" t="n">
+      <c r="B18" s="37" t="n">
         <f aca="false">B12-B17</f>
         <v>17.4515</v>
       </c>
@@ -6885,7 +7367,7 @@
       <c r="A19" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="B19" s="36" t="n">
+      <c r="B19" s="38" t="n">
         <f aca="false">B18/B5</f>
         <v>0.116382127375792</v>
       </c>
@@ -6943,7 +7425,7 @@
       <c r="A27" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="B27" s="34" t="n">
+      <c r="B27" s="36" t="n">
         <v>0.15</v>
       </c>
       <c r="C27" s="4" t="s">
@@ -7077,7 +7559,7 @@
       <c r="A41" s="4" t="s">
         <v>369</v>
       </c>
-      <c r="B41" s="34" t="n">
+      <c r="B41" s="36" t="n">
         <v>0.1</v>
       </c>
       <c r="C41" s="4" t="s">
@@ -7108,7 +7590,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7119,7 +7601,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:K23"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -7183,16 +7665,16 @@
       <c r="A5" s="4" t="s">
         <v>387</v>
       </c>
-      <c r="B5" s="37" t="n">
+      <c r="B5" s="39" t="n">
         <v>10000</v>
       </c>
-      <c r="C5" s="37" t="n">
+      <c r="C5" s="39" t="n">
         <v>200</v>
       </c>
       <c r="D5" s="6" t="n">
         <v>30000</v>
       </c>
-      <c r="E5" s="38" t="n">
+      <c r="E5" s="40" t="n">
         <f aca="false">C5/B5</f>
         <v>0.02</v>
       </c>
@@ -7221,16 +7703,16 @@
       <c r="A6" s="4" t="s">
         <v>389</v>
       </c>
-      <c r="B6" s="37" t="n">
+      <c r="B6" s="39" t="n">
         <v>12000</v>
       </c>
-      <c r="C6" s="37" t="n">
+      <c r="C6" s="39" t="n">
         <v>210</v>
       </c>
       <c r="D6" s="6" t="n">
         <v>31500</v>
       </c>
-      <c r="E6" s="38" t="n">
+      <c r="E6" s="40" t="n">
         <f aca="false">C6/B6</f>
         <v>0.0175</v>
       </c>
@@ -7254,7 +7736,7 @@
         <f aca="false">D6/D5-1</f>
         <v>0.05</v>
       </c>
-      <c r="K6" s="39" t="n">
+      <c r="K6" s="41" t="n">
         <f aca="false">(E6-E5)*100</f>
         <v>-0.25</v>
       </c>
@@ -7263,16 +7745,16 @@
       <c r="A7" s="4" t="s">
         <v>390</v>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="39" t="n">
         <v>15000</v>
       </c>
-      <c r="C7" s="37" t="n">
+      <c r="C7" s="39" t="n">
         <v>205</v>
       </c>
       <c r="D7" s="6" t="n">
         <v>30750</v>
       </c>
-      <c r="E7" s="38" t="n">
+      <c r="E7" s="40" t="n">
         <f aca="false">C7/B7</f>
         <v>0.0136666666666667</v>
       </c>
@@ -7296,7 +7778,7 @@
         <f aca="false">D7/D6-1</f>
         <v>-0.0238095238095238</v>
       </c>
-      <c r="K7" s="39" t="n">
+      <c r="K7" s="41" t="n">
         <f aca="false">(E7-E6)*100</f>
         <v>-0.383333333333333</v>
       </c>
@@ -7305,16 +7787,16 @@
       <c r="A8" s="4" t="s">
         <v>391</v>
       </c>
-      <c r="B8" s="37" t="n">
+      <c r="B8" s="39" t="n">
         <v>20000</v>
       </c>
-      <c r="C8" s="37" t="n">
+      <c r="C8" s="39" t="n">
         <v>210</v>
       </c>
       <c r="D8" s="6" t="n">
         <v>31500</v>
       </c>
-      <c r="E8" s="38" t="n">
+      <c r="E8" s="40" t="n">
         <f aca="false">C8/B8</f>
         <v>0.0105</v>
       </c>
@@ -7338,7 +7820,7 @@
         <f aca="false">D8/D7-1</f>
         <v>0.024390243902439</v>
       </c>
-      <c r="K8" s="39" t="n">
+      <c r="K8" s="41" t="n">
         <f aca="false">(E8-E7)*100</f>
         <v>-0.316666666666667</v>
       </c>
@@ -7347,27 +7829,27 @@
       <c r="A10" s="10" t="s">
         <v>392</v>
       </c>
-      <c r="B10" s="40" t="n">
+      <c r="B10" s="42" t="n">
         <f aca="false">B8/B5-1</f>
         <v>1</v>
       </c>
-      <c r="C10" s="40" t="n">
+      <c r="C10" s="42" t="n">
         <f aca="false">C8/C5-1</f>
         <v>0.05</v>
       </c>
-      <c r="D10" s="40" t="n">
+      <c r="D10" s="42" t="n">
         <f aca="false">D8/D5-1</f>
         <v>0.05</v>
       </c>
-      <c r="E10" s="40" t="n">
+      <c r="E10" s="42" t="n">
         <f aca="false">E8/E5-1</f>
         <v>-0.475</v>
       </c>
-      <c r="F10" s="40" t="n">
+      <c r="F10" s="42" t="n">
         <f aca="false">F8/F5-1</f>
         <v>0</v>
       </c>
-      <c r="G10" s="40" t="n">
+      <c r="G10" s="42" t="n">
         <f aca="false">G8/G5-1</f>
         <v>-0.475</v>
       </c>
@@ -7388,7 +7870,7 @@
         <f aca="false">D8-D5</f>
         <v>1500</v>
       </c>
-      <c r="E11" s="39" t="n">
+      <c r="E11" s="41" t="n">
         <f aca="false">(E8-E5)*100</f>
         <v>-0.95</v>
       </c>
@@ -7429,7 +7911,7 @@
       <c r="A17" s="4" t="s">
         <v>398</v>
       </c>
-      <c r="B17" s="38" t="n">
+      <c r="B17" s="40" t="n">
         <f aca="false">B15/B14</f>
         <v>0.001</v>
       </c>
@@ -7461,20 +7943,38 @@
         <v>28500</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" customFormat="false" ht="27.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="23" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="13"/>
+      <c r="F22" s="13"/>
+      <c r="G22" s="13"/>
+      <c r="H22" s="13"/>
+    </row>
+    <row r="23" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
         <v>403</v>
       </c>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="13"/>
+      <c r="F23" s="13"/>
+      <c r="G23" s="13"/>
+      <c r="H23" s="13"/>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A22:H22"/>
+    <mergeCell ref="A23:H23"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -7485,7 +7985,7 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
+    <pageSetUpPr fitToPage="true"/>
   </sheetPr>
   <dimension ref="A1:F19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
@@ -7518,7 +8018,7 @@
       <c r="A5" s="4" t="s">
         <v>408</v>
       </c>
-      <c r="B5" s="37" t="n">
+      <c r="B5" s="39" t="n">
         <v>10000</v>
       </c>
     </row>
@@ -7526,7 +8026,7 @@
       <c r="A6" s="4" t="s">
         <v>409</v>
       </c>
-      <c r="B6" s="37" t="n">
+      <c r="B6" s="39" t="n">
         <v>500</v>
       </c>
     </row>
@@ -7534,7 +8034,7 @@
       <c r="A7" s="4" t="s">
         <v>410</v>
       </c>
-      <c r="B7" s="37" t="n">
+      <c r="B7" s="39" t="n">
         <v>100</v>
       </c>
     </row>
@@ -7542,7 +8042,7 @@
       <c r="A8" s="4" t="s">
         <v>411</v>
       </c>
-      <c r="B8" s="37" t="n">
+      <c r="B8" s="39" t="n">
         <v>20</v>
       </c>
     </row>
@@ -7578,11 +8078,11 @@
         <f aca="false">B5</f>
         <v>10000</v>
       </c>
-      <c r="D11" s="36" t="n">
+      <c r="D11" s="38" t="n">
         <f aca="false">B11/C11</f>
         <v>0.05</v>
       </c>
-      <c r="E11" s="38" t="n">
+      <c r="E11" s="40" t="n">
         <f aca="false">1-D11</f>
         <v>0.95</v>
       </c>
@@ -7603,11 +8103,11 @@
         <f aca="false">B6</f>
         <v>500</v>
       </c>
-      <c r="D12" s="36" t="n">
+      <c r="D12" s="38" t="n">
         <f aca="false">B12/C12</f>
         <v>0.2</v>
       </c>
-      <c r="E12" s="38" t="n">
+      <c r="E12" s="40" t="n">
         <f aca="false">1-D12</f>
         <v>0.8</v>
       </c>
@@ -7628,11 +8128,11 @@
         <f aca="false">B7</f>
         <v>100</v>
       </c>
-      <c r="D13" s="36" t="n">
+      <c r="D13" s="38" t="n">
         <f aca="false">B13/C13</f>
         <v>0.2</v>
       </c>
-      <c r="E13" s="38" t="n">
+      <c r="E13" s="40" t="n">
         <f aca="false">1-D13</f>
         <v>0.8</v>
       </c>
@@ -7653,11 +8153,11 @@
         <f aca="false">B5</f>
         <v>10000</v>
       </c>
-      <c r="D14" s="36" t="n">
+      <c r="D14" s="38" t="n">
         <f aca="false">B14/C14</f>
         <v>0.002</v>
       </c>
-      <c r="E14" s="38" t="n">
+      <c r="E14" s="40" t="n">
         <f aca="false">1-D14</f>
         <v>0.998</v>
       </c>
@@ -7684,15 +8184,23 @@
         <v>OK</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="13.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
         <v>424</v>
       </c>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="13"/>
+      <c r="F19" s="13"/>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A19:F19"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="0" pageOrder="downThenOver" orientation="landscape" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>